<commit_message>
Resolve merge conflicts using remote version
</commit_message>
<xml_diff>
--- a/test_plan.xlsx
+++ b/test_plan.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OMEN\Documents\Eng. Raghad\DV\DV_project-claude-busy-turing-q1vwei\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OMEN\Documents\Eng. Raghad\DV\Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD10F78B-B97A-40B6-BE31-1358EC5A83E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32F7E3AF-B659-40D8-895F-4B6E698061C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{2A3F12D1-36D3-4428-BC65-043ACAAD9E53}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="320">
   <si>
     <t>Electrical and Computer Engineering Department</t>
   </si>
@@ -985,7 +985,7 @@
     <t>Run</t>
   </si>
   <si>
-    <t>Run with error</t>
+    <t>DUT Bug</t>
   </si>
 </sst>
 </file>
@@ -1294,7 +1294,16 @@
     <xf numFmtId="0" fontId="13" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="7" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1304,6 +1313,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1318,22 +1339,13 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1341,18 +1353,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1747,18 +1747,18 @@
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
-      <c r="J3" s="20" t="s">
+      <c r="J3" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="K3" s="20"/>
-      <c r="L3" s="20"/>
-      <c r="M3" s="20"/>
-      <c r="N3" s="20"/>
-      <c r="O3" s="20"/>
-      <c r="P3" s="20"/>
-      <c r="Q3" s="20"/>
-      <c r="R3" s="20"/>
-      <c r="S3" s="20"/>
+      <c r="K3" s="23"/>
+      <c r="L3" s="23"/>
+      <c r="M3" s="23"/>
+      <c r="N3" s="23"/>
+      <c r="O3" s="23"/>
+      <c r="P3" s="23"/>
+      <c r="Q3" s="23"/>
+      <c r="R3" s="23"/>
+      <c r="S3" s="23"/>
       <c r="T3" s="1"/>
       <c r="U3" s="1"/>
       <c r="V3" s="1"/>
@@ -1781,16 +1781,16 @@
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
-      <c r="J4" s="20"/>
-      <c r="K4" s="20"/>
-      <c r="L4" s="20"/>
-      <c r="M4" s="20"/>
-      <c r="N4" s="20"/>
-      <c r="O4" s="20"/>
-      <c r="P4" s="20"/>
-      <c r="Q4" s="20"/>
-      <c r="R4" s="20"/>
-      <c r="S4" s="20"/>
+      <c r="J4" s="23"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="23"/>
+      <c r="N4" s="23"/>
+      <c r="O4" s="23"/>
+      <c r="P4" s="23"/>
+      <c r="Q4" s="23"/>
+      <c r="R4" s="23"/>
+      <c r="S4" s="23"/>
       <c r="T4" s="1"/>
       <c r="U4" s="1"/>
       <c r="V4" s="1"/>
@@ -1813,18 +1813,18 @@
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
-      <c r="J5" s="20" t="s">
+      <c r="J5" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="K5" s="20"/>
-      <c r="L5" s="20"/>
-      <c r="M5" s="20"/>
-      <c r="N5" s="20"/>
-      <c r="O5" s="20"/>
-      <c r="P5" s="20"/>
-      <c r="Q5" s="20"/>
-      <c r="R5" s="20"/>
-      <c r="S5" s="20"/>
+      <c r="K5" s="23"/>
+      <c r="L5" s="23"/>
+      <c r="M5" s="23"/>
+      <c r="N5" s="23"/>
+      <c r="O5" s="23"/>
+      <c r="P5" s="23"/>
+      <c r="Q5" s="23"/>
+      <c r="R5" s="23"/>
+      <c r="S5" s="23"/>
       <c r="T5" s="1"/>
       <c r="U5" s="1"/>
       <c r="V5" s="1"/>
@@ -1847,16 +1847,16 @@
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
-      <c r="J6" s="20"/>
-      <c r="K6" s="20"/>
-      <c r="L6" s="20"/>
-      <c r="M6" s="20"/>
-      <c r="N6" s="20"/>
-      <c r="O6" s="20"/>
-      <c r="P6" s="20"/>
-      <c r="Q6" s="20"/>
-      <c r="R6" s="20"/>
-      <c r="S6" s="20"/>
+      <c r="J6" s="23"/>
+      <c r="K6" s="23"/>
+      <c r="L6" s="23"/>
+      <c r="M6" s="23"/>
+      <c r="N6" s="23"/>
+      <c r="O6" s="23"/>
+      <c r="P6" s="23"/>
+      <c r="Q6" s="23"/>
+      <c r="R6" s="23"/>
+      <c r="S6" s="23"/>
       <c r="T6" s="1"/>
       <c r="U6" s="1"/>
       <c r="V6" s="1"/>
@@ -1879,18 +1879,18 @@
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
-      <c r="J7" s="20" t="s">
+      <c r="J7" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="K7" s="20"/>
-      <c r="L7" s="20"/>
-      <c r="M7" s="20"/>
-      <c r="N7" s="20"/>
-      <c r="O7" s="20"/>
-      <c r="P7" s="20"/>
-      <c r="Q7" s="20"/>
-      <c r="R7" s="20"/>
-      <c r="S7" s="20"/>
+      <c r="K7" s="23"/>
+      <c r="L7" s="23"/>
+      <c r="M7" s="23"/>
+      <c r="N7" s="23"/>
+      <c r="O7" s="23"/>
+      <c r="P7" s="23"/>
+      <c r="Q7" s="23"/>
+      <c r="R7" s="23"/>
+      <c r="S7" s="23"/>
       <c r="T7" s="1"/>
       <c r="U7" s="1"/>
       <c r="V7" s="1"/>
@@ -1913,16 +1913,16 @@
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
-      <c r="J8" s="20"/>
-      <c r="K8" s="20"/>
-      <c r="L8" s="20"/>
-      <c r="M8" s="20"/>
-      <c r="N8" s="20"/>
-      <c r="O8" s="20"/>
-      <c r="P8" s="20"/>
-      <c r="Q8" s="20"/>
-      <c r="R8" s="20"/>
-      <c r="S8" s="20"/>
+      <c r="J8" s="23"/>
+      <c r="K8" s="23"/>
+      <c r="L8" s="23"/>
+      <c r="M8" s="23"/>
+      <c r="N8" s="23"/>
+      <c r="O8" s="23"/>
+      <c r="P8" s="23"/>
+      <c r="Q8" s="23"/>
+      <c r="R8" s="23"/>
+      <c r="S8" s="23"/>
       <c r="T8" s="1"/>
       <c r="U8" s="1"/>
       <c r="V8" s="1"/>
@@ -1945,18 +1945,18 @@
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
-      <c r="J9" s="20" t="s">
+      <c r="J9" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="K9" s="20"/>
-      <c r="L9" s="20"/>
-      <c r="M9" s="20"/>
-      <c r="N9" s="20"/>
-      <c r="O9" s="20"/>
-      <c r="P9" s="20"/>
-      <c r="Q9" s="20"/>
-      <c r="R9" s="20"/>
-      <c r="S9" s="20"/>
+      <c r="K9" s="23"/>
+      <c r="L9" s="23"/>
+      <c r="M9" s="23"/>
+      <c r="N9" s="23"/>
+      <c r="O9" s="23"/>
+      <c r="P9" s="23"/>
+      <c r="Q9" s="23"/>
+      <c r="R9" s="23"/>
+      <c r="S9" s="23"/>
       <c r="T9" s="1"/>
       <c r="U9" s="1"/>
       <c r="V9" s="1"/>
@@ -2075,18 +2075,18 @@
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
-      <c r="J13" s="20" t="s">
+      <c r="J13" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="K13" s="20"/>
-      <c r="L13" s="20"/>
-      <c r="M13" s="20"/>
-      <c r="N13" s="20"/>
-      <c r="O13" s="20"/>
-      <c r="P13" s="20"/>
-      <c r="Q13" s="20"/>
-      <c r="R13" s="20"/>
-      <c r="S13" s="20"/>
+      <c r="K13" s="23"/>
+      <c r="L13" s="23"/>
+      <c r="M13" s="23"/>
+      <c r="N13" s="23"/>
+      <c r="O13" s="23"/>
+      <c r="P13" s="23"/>
+      <c r="Q13" s="23"/>
+      <c r="R13" s="23"/>
+      <c r="S13" s="23"/>
       <c r="T13" s="1"/>
       <c r="U13" s="1"/>
       <c r="V13" s="1"/>
@@ -2109,16 +2109,16 @@
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
-      <c r="J14" s="20"/>
-      <c r="K14" s="20"/>
-      <c r="L14" s="20"/>
-      <c r="M14" s="20"/>
-      <c r="N14" s="20"/>
-      <c r="O14" s="20"/>
-      <c r="P14" s="20"/>
-      <c r="Q14" s="20"/>
-      <c r="R14" s="20"/>
-      <c r="S14" s="20"/>
+      <c r="J14" s="23"/>
+      <c r="K14" s="23"/>
+      <c r="L14" s="23"/>
+      <c r="M14" s="23"/>
+      <c r="N14" s="23"/>
+      <c r="O14" s="23"/>
+      <c r="P14" s="23"/>
+      <c r="Q14" s="23"/>
+      <c r="R14" s="23"/>
+      <c r="S14" s="23"/>
       <c r="T14" s="1"/>
       <c r="U14" s="1"/>
       <c r="V14" s="1"/>
@@ -2141,18 +2141,18 @@
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
-      <c r="J15" s="20" t="s">
+      <c r="J15" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="K15" s="20"/>
-      <c r="L15" s="20"/>
-      <c r="M15" s="20"/>
-      <c r="N15" s="20"/>
-      <c r="O15" s="20"/>
-      <c r="P15" s="20"/>
-      <c r="Q15" s="20"/>
-      <c r="R15" s="20"/>
-      <c r="S15" s="20"/>
+      <c r="K15" s="23"/>
+      <c r="L15" s="23"/>
+      <c r="M15" s="23"/>
+      <c r="N15" s="23"/>
+      <c r="O15" s="23"/>
+      <c r="P15" s="23"/>
+      <c r="Q15" s="23"/>
+      <c r="R15" s="23"/>
+      <c r="S15" s="23"/>
       <c r="T15" s="1"/>
       <c r="U15" s="1"/>
       <c r="V15" s="1"/>
@@ -2175,16 +2175,16 @@
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
-      <c r="J16" s="20"/>
-      <c r="K16" s="20"/>
-      <c r="L16" s="20"/>
-      <c r="M16" s="20"/>
-      <c r="N16" s="20"/>
-      <c r="O16" s="20"/>
-      <c r="P16" s="20"/>
-      <c r="Q16" s="20"/>
-      <c r="R16" s="20"/>
-      <c r="S16" s="20"/>
+      <c r="J16" s="23"/>
+      <c r="K16" s="23"/>
+      <c r="L16" s="23"/>
+      <c r="M16" s="23"/>
+      <c r="N16" s="23"/>
+      <c r="O16" s="23"/>
+      <c r="P16" s="23"/>
+      <c r="Q16" s="23"/>
+      <c r="R16" s="23"/>
+      <c r="S16" s="23"/>
       <c r="T16" s="1"/>
       <c r="U16" s="1"/>
       <c r="V16" s="1"/>
@@ -2207,18 +2207,18 @@
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
-      <c r="J17" s="20" t="s">
+      <c r="J17" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="K17" s="20"/>
-      <c r="L17" s="20"/>
-      <c r="M17" s="20"/>
-      <c r="N17" s="20"/>
-      <c r="O17" s="20"/>
-      <c r="P17" s="20"/>
-      <c r="Q17" s="20"/>
-      <c r="R17" s="20"/>
-      <c r="S17" s="20"/>
+      <c r="K17" s="23"/>
+      <c r="L17" s="23"/>
+      <c r="M17" s="23"/>
+      <c r="N17" s="23"/>
+      <c r="O17" s="23"/>
+      <c r="P17" s="23"/>
+      <c r="Q17" s="23"/>
+      <c r="R17" s="23"/>
+      <c r="S17" s="23"/>
       <c r="T17" s="1"/>
       <c r="U17" s="1"/>
       <c r="V17" s="1"/>
@@ -2241,16 +2241,16 @@
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
-      <c r="J18" s="20"/>
-      <c r="K18" s="20"/>
-      <c r="L18" s="20"/>
-      <c r="M18" s="20"/>
-      <c r="N18" s="20"/>
-      <c r="O18" s="20"/>
-      <c r="P18" s="20"/>
-      <c r="Q18" s="20"/>
-      <c r="R18" s="20"/>
-      <c r="S18" s="20"/>
+      <c r="J18" s="23"/>
+      <c r="K18" s="23"/>
+      <c r="L18" s="23"/>
+      <c r="M18" s="23"/>
+      <c r="N18" s="23"/>
+      <c r="O18" s="23"/>
+      <c r="P18" s="23"/>
+      <c r="Q18" s="23"/>
+      <c r="R18" s="23"/>
+      <c r="S18" s="23"/>
       <c r="T18" s="1"/>
       <c r="U18" s="1"/>
       <c r="V18" s="1"/>
@@ -2273,18 +2273,18 @@
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
-      <c r="J19" s="33" t="s">
+      <c r="J19" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="K19" s="33"/>
-      <c r="L19" s="33"/>
-      <c r="M19" s="33"/>
-      <c r="N19" s="33"/>
-      <c r="O19" s="33"/>
-      <c r="P19" s="33"/>
-      <c r="Q19" s="33"/>
-      <c r="R19" s="33"/>
-      <c r="S19" s="33"/>
+      <c r="K19" s="32"/>
+      <c r="L19" s="32"/>
+      <c r="M19" s="32"/>
+      <c r="N19" s="32"/>
+      <c r="O19" s="32"/>
+      <c r="P19" s="32"/>
+      <c r="Q19" s="32"/>
+      <c r="R19" s="32"/>
+      <c r="S19" s="32"/>
       <c r="T19" s="1"/>
       <c r="U19" s="1"/>
       <c r="V19" s="1"/>
@@ -2307,16 +2307,16 @@
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
-      <c r="J20" s="33"/>
-      <c r="K20" s="33"/>
-      <c r="L20" s="33"/>
-      <c r="M20" s="33"/>
-      <c r="N20" s="33"/>
-      <c r="O20" s="33"/>
-      <c r="P20" s="33"/>
-      <c r="Q20" s="33"/>
-      <c r="R20" s="33"/>
-      <c r="S20" s="33"/>
+      <c r="J20" s="32"/>
+      <c r="K20" s="32"/>
+      <c r="L20" s="32"/>
+      <c r="M20" s="32"/>
+      <c r="N20" s="32"/>
+      <c r="O20" s="32"/>
+      <c r="P20" s="32"/>
+      <c r="Q20" s="32"/>
+      <c r="R20" s="32"/>
+      <c r="S20" s="32"/>
       <c r="T20" s="1"/>
       <c r="U20" s="1"/>
       <c r="V20" s="1"/>
@@ -2339,16 +2339,16 @@
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
-      <c r="J21" s="33"/>
-      <c r="K21" s="33"/>
-      <c r="L21" s="33"/>
-      <c r="M21" s="33"/>
-      <c r="N21" s="33"/>
-      <c r="O21" s="33"/>
-      <c r="P21" s="33"/>
-      <c r="Q21" s="33"/>
-      <c r="R21" s="33"/>
-      <c r="S21" s="33"/>
+      <c r="J21" s="32"/>
+      <c r="K21" s="32"/>
+      <c r="L21" s="32"/>
+      <c r="M21" s="32"/>
+      <c r="N21" s="32"/>
+      <c r="O21" s="32"/>
+      <c r="P21" s="32"/>
+      <c r="Q21" s="32"/>
+      <c r="R21" s="32"/>
+      <c r="S21" s="32"/>
       <c r="T21" s="1"/>
       <c r="U21" s="1"/>
       <c r="V21" s="1"/>
@@ -2371,16 +2371,16 @@
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
-      <c r="J22" s="33"/>
-      <c r="K22" s="33"/>
-      <c r="L22" s="33"/>
-      <c r="M22" s="33"/>
-      <c r="N22" s="33"/>
-      <c r="O22" s="33"/>
-      <c r="P22" s="33"/>
-      <c r="Q22" s="33"/>
-      <c r="R22" s="33"/>
-      <c r="S22" s="33"/>
+      <c r="J22" s="32"/>
+      <c r="K22" s="32"/>
+      <c r="L22" s="32"/>
+      <c r="M22" s="32"/>
+      <c r="N22" s="32"/>
+      <c r="O22" s="32"/>
+      <c r="P22" s="32"/>
+      <c r="Q22" s="32"/>
+      <c r="R22" s="32"/>
+      <c r="S22" s="32"/>
       <c r="T22" s="1"/>
       <c r="U22" s="1"/>
       <c r="V22" s="1"/>
@@ -2531,18 +2531,18 @@
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
-      <c r="J27" s="20" t="s">
+      <c r="J27" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="K27" s="20"/>
-      <c r="L27" s="20"/>
-      <c r="M27" s="20"/>
-      <c r="N27" s="20"/>
-      <c r="O27" s="20"/>
-      <c r="P27" s="20"/>
-      <c r="Q27" s="20"/>
-      <c r="R27" s="20"/>
-      <c r="S27" s="20"/>
+      <c r="K27" s="23"/>
+      <c r="L27" s="23"/>
+      <c r="M27" s="23"/>
+      <c r="N27" s="23"/>
+      <c r="O27" s="23"/>
+      <c r="P27" s="23"/>
+      <c r="Q27" s="23"/>
+      <c r="R27" s="23"/>
+      <c r="S27" s="23"/>
       <c r="T27" s="1"/>
       <c r="U27" s="1"/>
       <c r="V27" s="1"/>
@@ -2565,16 +2565,16 @@
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
-      <c r="J28" s="20"/>
-      <c r="K28" s="20"/>
-      <c r="L28" s="20"/>
-      <c r="M28" s="20"/>
-      <c r="N28" s="20"/>
-      <c r="O28" s="20"/>
-      <c r="P28" s="20"/>
-      <c r="Q28" s="20"/>
-      <c r="R28" s="20"/>
-      <c r="S28" s="20"/>
+      <c r="J28" s="23"/>
+      <c r="K28" s="23"/>
+      <c r="L28" s="23"/>
+      <c r="M28" s="23"/>
+      <c r="N28" s="23"/>
+      <c r="O28" s="23"/>
+      <c r="P28" s="23"/>
+      <c r="Q28" s="23"/>
+      <c r="R28" s="23"/>
+      <c r="S28" s="23"/>
       <c r="T28" s="1"/>
       <c r="U28" s="1"/>
       <c r="V28" s="1"/>
@@ -2597,22 +2597,22 @@
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
-      <c r="J29" s="27" t="s">
+      <c r="J29" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="K29" s="31"/>
-      <c r="L29" s="31"/>
-      <c r="M29" s="31"/>
-      <c r="N29" s="31"/>
-      <c r="O29" s="28"/>
-      <c r="P29" s="27" t="s">
+      <c r="K29" s="35"/>
+      <c r="L29" s="35"/>
+      <c r="M29" s="35"/>
+      <c r="N29" s="35"/>
+      <c r="O29" s="25"/>
+      <c r="P29" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="Q29" s="28"/>
-      <c r="R29" s="27" t="s">
+      <c r="Q29" s="25"/>
+      <c r="R29" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="S29" s="28"/>
+      <c r="S29" s="25"/>
       <c r="T29" s="1"/>
       <c r="U29" s="1"/>
       <c r="V29" s="1"/>
@@ -2635,16 +2635,16 @@
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
-      <c r="J30" s="29"/>
-      <c r="K30" s="32"/>
-      <c r="L30" s="32"/>
-      <c r="M30" s="32"/>
-      <c r="N30" s="32"/>
-      <c r="O30" s="30"/>
-      <c r="P30" s="29"/>
-      <c r="Q30" s="30"/>
-      <c r="R30" s="29"/>
-      <c r="S30" s="30"/>
+      <c r="J30" s="26"/>
+      <c r="K30" s="36"/>
+      <c r="L30" s="36"/>
+      <c r="M30" s="36"/>
+      <c r="N30" s="36"/>
+      <c r="O30" s="27"/>
+      <c r="P30" s="26"/>
+      <c r="Q30" s="27"/>
+      <c r="R30" s="26"/>
+      <c r="S30" s="27"/>
       <c r="T30" s="1"/>
       <c r="U30" s="1"/>
       <c r="V30" s="1"/>
@@ -2667,22 +2667,22 @@
       <c r="G31" s="1"/>
       <c r="H31" s="1"/>
       <c r="I31" s="1"/>
-      <c r="J31" s="21" t="s">
+      <c r="J31" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="K31" s="25"/>
-      <c r="L31" s="25"/>
-      <c r="M31" s="25"/>
-      <c r="N31" s="25"/>
-      <c r="O31" s="22"/>
-      <c r="P31" s="21">
+      <c r="K31" s="33"/>
+      <c r="L31" s="33"/>
+      <c r="M31" s="33"/>
+      <c r="N31" s="33"/>
+      <c r="O31" s="29"/>
+      <c r="P31" s="28">
         <v>1191612</v>
       </c>
-      <c r="Q31" s="22"/>
-      <c r="R31" s="21">
+      <c r="Q31" s="29"/>
+      <c r="R31" s="28">
         <v>2</v>
       </c>
-      <c r="S31" s="22"/>
+      <c r="S31" s="29"/>
       <c r="T31" s="1"/>
       <c r="U31" s="1"/>
       <c r="V31" s="1"/>
@@ -2705,16 +2705,16 @@
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
       <c r="I32" s="3"/>
-      <c r="J32" s="23"/>
-      <c r="K32" s="26"/>
-      <c r="L32" s="26"/>
-      <c r="M32" s="26"/>
-      <c r="N32" s="26"/>
-      <c r="O32" s="24"/>
-      <c r="P32" s="23"/>
-      <c r="Q32" s="24"/>
-      <c r="R32" s="23"/>
-      <c r="S32" s="24"/>
+      <c r="J32" s="30"/>
+      <c r="K32" s="34"/>
+      <c r="L32" s="34"/>
+      <c r="M32" s="34"/>
+      <c r="N32" s="34"/>
+      <c r="O32" s="31"/>
+      <c r="P32" s="30"/>
+      <c r="Q32" s="31"/>
+      <c r="R32" s="30"/>
+      <c r="S32" s="31"/>
       <c r="T32" s="3"/>
       <c r="U32" s="3"/>
       <c r="V32" s="3"/>
@@ -2737,22 +2737,22 @@
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
       <c r="I33" s="3"/>
-      <c r="J33" s="21" t="s">
+      <c r="J33" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="K33" s="25"/>
-      <c r="L33" s="25"/>
-      <c r="M33" s="25"/>
-      <c r="N33" s="25"/>
-      <c r="O33" s="22"/>
-      <c r="P33" s="21">
+      <c r="K33" s="33"/>
+      <c r="L33" s="33"/>
+      <c r="M33" s="33"/>
+      <c r="N33" s="33"/>
+      <c r="O33" s="29"/>
+      <c r="P33" s="28">
         <v>1212214</v>
       </c>
-      <c r="Q33" s="22"/>
-      <c r="R33" s="21">
+      <c r="Q33" s="29"/>
+      <c r="R33" s="28">
         <v>1</v>
       </c>
-      <c r="S33" s="22"/>
+      <c r="S33" s="29"/>
       <c r="T33" s="3"/>
       <c r="U33" s="3"/>
       <c r="V33" s="3"/>
@@ -2775,16 +2775,16 @@
       <c r="G34" s="3"/>
       <c r="H34" s="3"/>
       <c r="I34" s="3"/>
-      <c r="J34" s="23"/>
-      <c r="K34" s="26"/>
-      <c r="L34" s="26"/>
-      <c r="M34" s="26"/>
-      <c r="N34" s="26"/>
-      <c r="O34" s="24"/>
-      <c r="P34" s="23"/>
-      <c r="Q34" s="24"/>
-      <c r="R34" s="23"/>
-      <c r="S34" s="24"/>
+      <c r="J34" s="30"/>
+      <c r="K34" s="34"/>
+      <c r="L34" s="34"/>
+      <c r="M34" s="34"/>
+      <c r="N34" s="34"/>
+      <c r="O34" s="31"/>
+      <c r="P34" s="30"/>
+      <c r="Q34" s="31"/>
+      <c r="R34" s="30"/>
+      <c r="S34" s="31"/>
       <c r="T34" s="3"/>
       <c r="U34" s="3"/>
       <c r="V34" s="3"/>
@@ -2807,22 +2807,22 @@
       <c r="G35" s="3"/>
       <c r="H35" s="3"/>
       <c r="I35" s="3"/>
-      <c r="J35" s="21" t="s">
+      <c r="J35" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="K35" s="25"/>
-      <c r="L35" s="25"/>
-      <c r="M35" s="25"/>
-      <c r="N35" s="25"/>
-      <c r="O35" s="22"/>
-      <c r="P35" s="21">
+      <c r="K35" s="33"/>
+      <c r="L35" s="33"/>
+      <c r="M35" s="33"/>
+      <c r="N35" s="33"/>
+      <c r="O35" s="29"/>
+      <c r="P35" s="28">
         <v>1221082</v>
       </c>
-      <c r="Q35" s="22"/>
-      <c r="R35" s="21">
+      <c r="Q35" s="29"/>
+      <c r="R35" s="28">
         <v>1</v>
       </c>
-      <c r="S35" s="22"/>
+      <c r="S35" s="29"/>
       <c r="T35" s="3"/>
       <c r="U35" s="3"/>
       <c r="V35" s="3"/>
@@ -2845,16 +2845,16 @@
       <c r="G36" s="3"/>
       <c r="H36" s="3"/>
       <c r="I36" s="3"/>
-      <c r="J36" s="23"/>
-      <c r="K36" s="26"/>
-      <c r="L36" s="26"/>
-      <c r="M36" s="26"/>
-      <c r="N36" s="26"/>
-      <c r="O36" s="24"/>
-      <c r="P36" s="23"/>
-      <c r="Q36" s="24"/>
-      <c r="R36" s="23"/>
-      <c r="S36" s="24"/>
+      <c r="J36" s="30"/>
+      <c r="K36" s="34"/>
+      <c r="L36" s="34"/>
+      <c r="M36" s="34"/>
+      <c r="N36" s="34"/>
+      <c r="O36" s="31"/>
+      <c r="P36" s="30"/>
+      <c r="Q36" s="31"/>
+      <c r="R36" s="30"/>
+      <c r="S36" s="31"/>
       <c r="T36" s="3"/>
       <c r="U36" s="3"/>
       <c r="V36" s="3"/>
@@ -2877,22 +2877,22 @@
       <c r="G37" s="3"/>
       <c r="H37" s="3"/>
       <c r="I37" s="3"/>
-      <c r="J37" s="21" t="s">
+      <c r="J37" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="K37" s="25"/>
-      <c r="L37" s="25"/>
-      <c r="M37" s="25"/>
-      <c r="N37" s="25"/>
-      <c r="O37" s="22"/>
-      <c r="P37" s="21">
+      <c r="K37" s="33"/>
+      <c r="L37" s="33"/>
+      <c r="M37" s="33"/>
+      <c r="N37" s="33"/>
+      <c r="O37" s="29"/>
+      <c r="P37" s="28">
         <v>1222275</v>
       </c>
-      <c r="Q37" s="22"/>
-      <c r="R37" s="21">
+      <c r="Q37" s="29"/>
+      <c r="R37" s="28">
         <v>2</v>
       </c>
-      <c r="S37" s="22"/>
+      <c r="S37" s="29"/>
       <c r="T37" s="3"/>
       <c r="U37" s="3"/>
       <c r="V37" s="3"/>
@@ -2915,16 +2915,16 @@
       <c r="G38" s="3"/>
       <c r="H38" s="3"/>
       <c r="I38" s="3"/>
-      <c r="J38" s="23"/>
-      <c r="K38" s="26"/>
-      <c r="L38" s="26"/>
-      <c r="M38" s="26"/>
-      <c r="N38" s="26"/>
-      <c r="O38" s="24"/>
-      <c r="P38" s="23"/>
-      <c r="Q38" s="24"/>
-      <c r="R38" s="23"/>
-      <c r="S38" s="24"/>
+      <c r="J38" s="30"/>
+      <c r="K38" s="34"/>
+      <c r="L38" s="34"/>
+      <c r="M38" s="34"/>
+      <c r="N38" s="34"/>
+      <c r="O38" s="31"/>
+      <c r="P38" s="30"/>
+      <c r="Q38" s="31"/>
+      <c r="R38" s="30"/>
+      <c r="S38" s="31"/>
       <c r="T38" s="3"/>
       <c r="U38" s="3"/>
       <c r="V38" s="3"/>
@@ -3011,18 +3011,18 @@
       <c r="G41" s="3"/>
       <c r="H41" s="3"/>
       <c r="I41" s="3"/>
-      <c r="J41" s="20" t="s">
+      <c r="J41" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="K41" s="20"/>
-      <c r="L41" s="20"/>
-      <c r="M41" s="20"/>
-      <c r="N41" s="20"/>
-      <c r="O41" s="20"/>
-      <c r="P41" s="20"/>
-      <c r="Q41" s="20"/>
-      <c r="R41" s="20"/>
-      <c r="S41" s="20"/>
+      <c r="K41" s="23"/>
+      <c r="L41" s="23"/>
+      <c r="M41" s="23"/>
+      <c r="N41" s="23"/>
+      <c r="O41" s="23"/>
+      <c r="P41" s="23"/>
+      <c r="Q41" s="23"/>
+      <c r="R41" s="23"/>
+      <c r="S41" s="23"/>
       <c r="T41" s="3"/>
       <c r="U41" s="3"/>
       <c r="V41" s="3"/>
@@ -3045,16 +3045,16 @@
       <c r="G42" s="3"/>
       <c r="H42" s="3"/>
       <c r="I42" s="3"/>
-      <c r="J42" s="20"/>
-      <c r="K42" s="20"/>
-      <c r="L42" s="20"/>
-      <c r="M42" s="20"/>
-      <c r="N42" s="20"/>
-      <c r="O42" s="20"/>
-      <c r="P42" s="20"/>
-      <c r="Q42" s="20"/>
-      <c r="R42" s="20"/>
-      <c r="S42" s="20"/>
+      <c r="J42" s="23"/>
+      <c r="K42" s="23"/>
+      <c r="L42" s="23"/>
+      <c r="M42" s="23"/>
+      <c r="N42" s="23"/>
+      <c r="O42" s="23"/>
+      <c r="P42" s="23"/>
+      <c r="Q42" s="23"/>
+      <c r="R42" s="23"/>
+      <c r="S42" s="23"/>
       <c r="T42" s="3"/>
       <c r="U42" s="3"/>
       <c r="V42" s="3"/>
@@ -3101,9 +3101,6 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="J17:S18"/>
-    <mergeCell ref="J19:S22"/>
-    <mergeCell ref="J27:S28"/>
     <mergeCell ref="J41:S42"/>
     <mergeCell ref="R35:S36"/>
     <mergeCell ref="J37:O38"/>
@@ -3117,15 +3114,18 @@
     <mergeCell ref="J35:O36"/>
     <mergeCell ref="P35:Q36"/>
     <mergeCell ref="P37:Q38"/>
-    <mergeCell ref="P29:Q30"/>
     <mergeCell ref="P31:Q32"/>
     <mergeCell ref="P33:Q34"/>
     <mergeCell ref="J5:S6"/>
     <mergeCell ref="J7:S8"/>
+    <mergeCell ref="J17:S18"/>
+    <mergeCell ref="J19:S22"/>
+    <mergeCell ref="J27:S28"/>
     <mergeCell ref="J3:S4"/>
     <mergeCell ref="J13:S14"/>
     <mergeCell ref="J15:S16"/>
     <mergeCell ref="J9:S9"/>
+    <mergeCell ref="P29:Q30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3133,7 +3133,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{758D3593-4783-47CC-8D9F-31D13BF080F4}">
-  <dimension ref="A1:J62"/>
+  <dimension ref="A1:K62"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="20.7109375" customWidth="1"/>
@@ -3143,7 +3143,7 @@
     <col min="10" max="11" width="42.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>17</v>
       </c>
@@ -3171,25 +3171,25 @@
       <c r="I1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="J1" s="34" t="s">
+      <c r="J1" s="17" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+    <row r="2" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="21" t="s">
         <v>293</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-    </row>
-    <row r="3" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+    </row>
+    <row r="3" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>26</v>
       </c>
@@ -3217,11 +3217,11 @@
       <c r="I3" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="35" t="s">
+      <c r="J3" s="18" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>26</v>
       </c>
@@ -3249,9 +3249,9 @@
       <c r="I4" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="J4" s="36"/>
-    </row>
-    <row r="5" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J4" s="19"/>
+    </row>
+    <row r="5" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>26</v>
       </c>
@@ -3279,9 +3279,9 @@
       <c r="I5" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="J5" s="35"/>
-    </row>
-    <row r="6" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J5" s="18"/>
+    </row>
+    <row r="6" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>26</v>
       </c>
@@ -3309,23 +3309,23 @@
       <c r="I6" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="J6" s="36"/>
-    </row>
-    <row r="7" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="18" t="s">
+      <c r="J6" s="19"/>
+    </row>
+    <row r="7" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="21" t="s">
         <v>294</v>
       </c>
-      <c r="B7" s="19"/>
-      <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="19"/>
-      <c r="F7" s="19"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="19"/>
-      <c r="J7" s="19"/>
-    </row>
-    <row r="8" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="22"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="22"/>
+      <c r="I7" s="22"/>
+      <c r="J7" s="22"/>
+    </row>
+    <row r="8" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>47</v>
       </c>
@@ -3353,9 +3353,9 @@
       <c r="I8" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="J8" s="35"/>
-    </row>
-    <row r="9" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J8" s="18"/>
+    </row>
+    <row r="9" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>47</v>
       </c>
@@ -3383,9 +3383,9 @@
       <c r="I9" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="J9" s="36"/>
-    </row>
-    <row r="10" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J9" s="19"/>
+    </row>
+    <row r="10" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>47</v>
       </c>
@@ -3413,23 +3413,23 @@
       <c r="I10" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="J10" s="35"/>
-    </row>
-    <row r="11" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="18" t="s">
+      <c r="J10" s="18"/>
+    </row>
+    <row r="11" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="21" t="s">
         <v>295</v>
       </c>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19"/>
-      <c r="H11" s="19"/>
-      <c r="I11" s="19"/>
-      <c r="J11" s="19"/>
-    </row>
-    <row r="12" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="22"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
+      <c r="G11" s="22"/>
+      <c r="H11" s="22"/>
+      <c r="I11" s="22"/>
+      <c r="J11" s="22"/>
+    </row>
+    <row r="12" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>63</v>
       </c>
@@ -3451,15 +3451,15 @@
       <c r="G12" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="H12" s="8" t="s">
-        <v>32</v>
+      <c r="H12" s="15" t="s">
+        <v>318</v>
       </c>
       <c r="I12" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="J12" s="35"/>
-    </row>
-    <row r="13" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J12" s="18"/>
+    </row>
+    <row r="13" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>63</v>
       </c>
@@ -3481,15 +3481,15 @@
       <c r="G13" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="H13" s="12" t="s">
-        <v>32</v>
+      <c r="H13" s="15" t="s">
+        <v>318</v>
       </c>
       <c r="I13" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="J13" s="36"/>
-    </row>
-    <row r="14" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J13" s="19"/>
+    </row>
+    <row r="14" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>63</v>
       </c>
@@ -3511,15 +3511,18 @@
       <c r="G14" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="H14" s="8" t="s">
-        <v>32</v>
+      <c r="H14" s="15" t="s">
+        <v>318</v>
       </c>
       <c r="I14" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="J14" s="35"/>
-    </row>
-    <row r="15" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J14" s="18"/>
+      <c r="K14" s="20" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>63</v>
       </c>
@@ -3541,15 +3544,18 @@
       <c r="G15" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="H15" s="12" t="s">
-        <v>32</v>
+      <c r="H15" s="15" t="s">
+        <v>318</v>
       </c>
       <c r="I15" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="J15" s="36"/>
-    </row>
-    <row r="16" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J15" s="19"/>
+      <c r="K15" s="20" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>63</v>
       </c>
@@ -3571,29 +3577,32 @@
       <c r="G16" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="H16" s="8" t="s">
-        <v>32</v>
+      <c r="H16" s="15" t="s">
+        <v>318</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="J16" s="35"/>
-    </row>
-    <row r="17" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="18" t="s">
+      <c r="J16" s="18"/>
+      <c r="K16" s="20" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="21" t="s">
         <v>297</v>
       </c>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="19"/>
-      <c r="J17" s="19"/>
-    </row>
-    <row r="18" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="22"/>
+      <c r="F17" s="22"/>
+      <c r="G17" s="22"/>
+      <c r="H17" s="22"/>
+      <c r="I17" s="22"/>
+      <c r="J17" s="22"/>
+    </row>
+    <row r="18" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>88</v>
       </c>
@@ -3621,9 +3630,9 @@
       <c r="I18" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="J18" s="35"/>
-    </row>
-    <row r="19" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J18" s="18"/>
+    </row>
+    <row r="19" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>88</v>
       </c>
@@ -3645,29 +3654,32 @@
       <c r="G19" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="H19" s="17" t="s">
-        <v>319</v>
+      <c r="H19" s="15" t="s">
+        <v>318</v>
       </c>
       <c r="I19" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="J19" s="36"/>
-    </row>
-    <row r="20" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="18" t="s">
+      <c r="J19" s="19"/>
+      <c r="K19" s="20" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="21" t="s">
         <v>296</v>
       </c>
-      <c r="B20" s="19"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19"/>
-      <c r="H20" s="19"/>
-      <c r="I20" s="19"/>
-      <c r="J20" s="19"/>
-    </row>
-    <row r="21" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="22"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="22"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="22"/>
+      <c r="I20" s="22"/>
+      <c r="J20" s="22"/>
+    </row>
+    <row r="21" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>98</v>
       </c>
@@ -3695,11 +3707,11 @@
       <c r="I21" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="J21" s="35" t="s">
+      <c r="J21" s="18" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>98</v>
       </c>
@@ -3727,9 +3739,9 @@
       <c r="I22" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="J22" s="36"/>
-    </row>
-    <row r="23" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J22" s="19"/>
+    </row>
+    <row r="23" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>98</v>
       </c>
@@ -3757,9 +3769,9 @@
       <c r="I23" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="J23" s="35"/>
-    </row>
-    <row r="24" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J23" s="18"/>
+    </row>
+    <row r="24" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
         <v>98</v>
       </c>
@@ -3787,9 +3799,9 @@
       <c r="I24" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="J24" s="36"/>
-    </row>
-    <row r="25" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J24" s="19"/>
+    </row>
+    <row r="25" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>98</v>
       </c>
@@ -3817,9 +3829,9 @@
       <c r="I25" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="J25" s="35"/>
-    </row>
-    <row r="26" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J25" s="18"/>
+    </row>
+    <row r="26" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
         <v>98</v>
       </c>
@@ -3847,9 +3859,9 @@
       <c r="I26" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="J26" s="36"/>
-    </row>
-    <row r="27" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J26" s="19"/>
+    </row>
+    <row r="27" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>98</v>
       </c>
@@ -3877,9 +3889,9 @@
       <c r="I27" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="J27" s="35"/>
-    </row>
-    <row r="28" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J27" s="18"/>
+    </row>
+    <row r="28" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
         <v>98</v>
       </c>
@@ -3907,9 +3919,9 @@
       <c r="I28" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="J28" s="36"/>
-    </row>
-    <row r="29" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J28" s="19"/>
+    </row>
+    <row r="29" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>98</v>
       </c>
@@ -3937,25 +3949,25 @@
       <c r="I29" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="J29" s="35" t="s">
+      <c r="J29" s="18" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="18" t="s">
+    <row r="30" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="21" t="s">
         <v>299</v>
       </c>
-      <c r="B30" s="19"/>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="19"/>
-      <c r="G30" s="19"/>
-      <c r="H30" s="19"/>
-      <c r="I30" s="19"/>
-      <c r="J30" s="19"/>
-    </row>
-    <row r="31" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="22"/>
+      <c r="C30" s="22"/>
+      <c r="D30" s="22"/>
+      <c r="E30" s="22"/>
+      <c r="F30" s="22"/>
+      <c r="G30" s="22"/>
+      <c r="H30" s="22"/>
+      <c r="I30" s="22"/>
+      <c r="J30" s="22"/>
+    </row>
+    <row r="31" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>134</v>
       </c>
@@ -3983,9 +3995,9 @@
       <c r="I31" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="J31" s="35"/>
-    </row>
-    <row r="32" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J31" s="18"/>
+    </row>
+    <row r="32" spans="1:11" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="9" t="s">
         <v>134</v>
       </c>
@@ -4013,7 +4025,7 @@
       <c r="I32" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="J32" s="36"/>
+      <c r="J32" s="19"/>
     </row>
     <row r="33" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
@@ -4043,7 +4055,7 @@
       <c r="I33" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="J33" s="35"/>
+      <c r="J33" s="18"/>
     </row>
     <row r="34" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="9" t="s">
@@ -4073,21 +4085,21 @@
       <c r="I34" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="J34" s="36"/>
+      <c r="J34" s="19"/>
     </row>
     <row r="35" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="18" t="s">
+      <c r="A35" s="21" t="s">
         <v>298</v>
       </c>
-      <c r="B35" s="19"/>
-      <c r="C35" s="19"/>
-      <c r="D35" s="19"/>
-      <c r="E35" s="19"/>
-      <c r="F35" s="19"/>
-      <c r="G35" s="19"/>
-      <c r="H35" s="19"/>
-      <c r="I35" s="19"/>
-      <c r="J35" s="19"/>
+      <c r="B35" s="22"/>
+      <c r="C35" s="22"/>
+      <c r="D35" s="22"/>
+      <c r="E35" s="22"/>
+      <c r="F35" s="22"/>
+      <c r="G35" s="22"/>
+      <c r="H35" s="22"/>
+      <c r="I35" s="22"/>
+      <c r="J35" s="22"/>
     </row>
     <row r="36" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
@@ -4117,7 +4129,7 @@
       <c r="I36" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="J36" s="35"/>
+      <c r="J36" s="18"/>
     </row>
     <row r="37" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="9" t="s">
@@ -4147,7 +4159,7 @@
       <c r="I37" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="J37" s="36"/>
+      <c r="J37" s="19"/>
     </row>
     <row r="38" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
@@ -4177,7 +4189,7 @@
       <c r="I38" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="J38" s="35"/>
+      <c r="J38" s="18"/>
     </row>
     <row r="39" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="9" t="s">
@@ -4207,7 +4219,7 @@
       <c r="I39" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="J39" s="36"/>
+      <c r="J39" s="19"/>
     </row>
     <row r="40" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
@@ -4237,23 +4249,23 @@
       <c r="I40" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="J40" s="35" t="s">
+      <c r="J40" s="18" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="18" t="s">
+      <c r="A41" s="21" t="s">
         <v>300</v>
       </c>
-      <c r="B41" s="19"/>
-      <c r="C41" s="19"/>
-      <c r="D41" s="19"/>
-      <c r="E41" s="19"/>
-      <c r="F41" s="19"/>
-      <c r="G41" s="19"/>
-      <c r="H41" s="19"/>
-      <c r="I41" s="19"/>
-      <c r="J41" s="19"/>
+      <c r="B41" s="22"/>
+      <c r="C41" s="22"/>
+      <c r="D41" s="22"/>
+      <c r="E41" s="22"/>
+      <c r="F41" s="22"/>
+      <c r="G41" s="22"/>
+      <c r="H41" s="22"/>
+      <c r="I41" s="22"/>
+      <c r="J41" s="22"/>
     </row>
     <row r="42" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
@@ -4283,7 +4295,7 @@
       <c r="I42" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="J42" s="35" t="s">
+      <c r="J42" s="18" t="s">
         <v>180</v>
       </c>
     </row>
@@ -4315,7 +4327,7 @@
       <c r="I43" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="J43" s="36" t="s">
+      <c r="J43" s="19" t="s">
         <v>186</v>
       </c>
     </row>
@@ -4347,7 +4359,7 @@
       <c r="I44" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="J44" s="35"/>
+      <c r="J44" s="18"/>
     </row>
     <row r="45" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="9" t="s">
@@ -4377,21 +4389,21 @@
       <c r="I45" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="J45" s="36"/>
+      <c r="J45" s="19"/>
     </row>
     <row r="46" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="18" t="s">
+      <c r="A46" s="21" t="s">
         <v>316</v>
       </c>
-      <c r="B46" s="19"/>
-      <c r="C46" s="19"/>
-      <c r="D46" s="19"/>
-      <c r="E46" s="19"/>
-      <c r="F46" s="19"/>
-      <c r="G46" s="19"/>
-      <c r="H46" s="19"/>
-      <c r="I46" s="19"/>
-      <c r="J46" s="19"/>
+      <c r="B46" s="22"/>
+      <c r="C46" s="22"/>
+      <c r="D46" s="22"/>
+      <c r="E46" s="22"/>
+      <c r="F46" s="22"/>
+      <c r="G46" s="22"/>
+      <c r="H46" s="22"/>
+      <c r="I46" s="22"/>
+      <c r="J46" s="22"/>
     </row>
     <row r="47" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
@@ -4421,7 +4433,7 @@
       <c r="I47" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="J47" s="35"/>
+      <c r="J47" s="18"/>
     </row>
     <row r="48" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="9" t="s">
@@ -4451,7 +4463,7 @@
       <c r="I48" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="J48" s="36"/>
+      <c r="J48" s="19"/>
     </row>
     <row r="49" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
@@ -4481,7 +4493,7 @@
       <c r="I49" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="J49" s="35"/>
+      <c r="J49" s="18"/>
     </row>
     <row r="50" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="9" t="s">
@@ -4511,7 +4523,7 @@
       <c r="I50" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="J50" s="36"/>
+      <c r="J50" s="19"/>
     </row>
     <row r="51" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
@@ -4541,7 +4553,7 @@
       <c r="I51" s="5" t="s">
         <v>200</v>
       </c>
-      <c r="J51" s="35" t="s">
+      <c r="J51" s="18" t="s">
         <v>217</v>
       </c>
     </row>
@@ -4573,21 +4585,21 @@
       <c r="I52" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="J52" s="36"/>
+      <c r="J52" s="19"/>
     </row>
     <row r="53" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="18" t="s">
+      <c r="A53" s="21" t="s">
         <v>301</v>
       </c>
-      <c r="B53" s="19"/>
-      <c r="C53" s="19"/>
-      <c r="D53" s="19"/>
-      <c r="E53" s="19"/>
-      <c r="F53" s="19"/>
-      <c r="G53" s="19"/>
-      <c r="H53" s="19"/>
-      <c r="I53" s="19"/>
-      <c r="J53" s="19"/>
+      <c r="B53" s="22"/>
+      <c r="C53" s="22"/>
+      <c r="D53" s="22"/>
+      <c r="E53" s="22"/>
+      <c r="F53" s="22"/>
+      <c r="G53" s="22"/>
+      <c r="H53" s="22"/>
+      <c r="I53" s="22"/>
+      <c r="J53" s="22"/>
     </row>
     <row r="54" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
@@ -4617,7 +4629,7 @@
       <c r="I54" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="J54" s="35"/>
+      <c r="J54" s="18"/>
     </row>
     <row r="55" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="9" t="s">
@@ -4647,7 +4659,7 @@
       <c r="I55" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="J55" s="36" t="s">
+      <c r="J55" s="19" t="s">
         <v>230</v>
       </c>
     </row>
@@ -4679,21 +4691,21 @@
       <c r="I56" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="J56" s="35"/>
+      <c r="J56" s="18"/>
     </row>
     <row r="57" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="18" t="s">
+      <c r="A57" s="21" t="s">
         <v>302</v>
       </c>
-      <c r="B57" s="19"/>
-      <c r="C57" s="19"/>
-      <c r="D57" s="19"/>
-      <c r="E57" s="19"/>
-      <c r="F57" s="19"/>
-      <c r="G57" s="19"/>
-      <c r="H57" s="19"/>
-      <c r="I57" s="19"/>
-      <c r="J57" s="19"/>
+      <c r="B57" s="22"/>
+      <c r="C57" s="22"/>
+      <c r="D57" s="22"/>
+      <c r="E57" s="22"/>
+      <c r="F57" s="22"/>
+      <c r="G57" s="22"/>
+      <c r="H57" s="22"/>
+      <c r="I57" s="22"/>
+      <c r="J57" s="22"/>
     </row>
     <row r="58" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
@@ -4723,7 +4735,7 @@
       <c r="I58" s="5" t="s">
         <v>240</v>
       </c>
-      <c r="J58" s="35"/>
+      <c r="J58" s="18"/>
     </row>
     <row r="59" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="9" t="s">
@@ -4753,21 +4765,21 @@
       <c r="I59" s="9" t="s">
         <v>240</v>
       </c>
-      <c r="J59" s="36"/>
+      <c r="J59" s="19"/>
     </row>
     <row r="60" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="18" t="s">
+      <c r="A60" s="21" t="s">
         <v>317</v>
       </c>
-      <c r="B60" s="19"/>
-      <c r="C60" s="19"/>
-      <c r="D60" s="19"/>
-      <c r="E60" s="19"/>
-      <c r="F60" s="19"/>
-      <c r="G60" s="19"/>
-      <c r="H60" s="19"/>
-      <c r="I60" s="19"/>
-      <c r="J60" s="19"/>
+      <c r="B60" s="22"/>
+      <c r="C60" s="22"/>
+      <c r="D60" s="22"/>
+      <c r="E60" s="22"/>
+      <c r="F60" s="22"/>
+      <c r="G60" s="22"/>
+      <c r="H60" s="22"/>
+      <c r="I60" s="22"/>
+      <c r="J60" s="22"/>
     </row>
     <row r="61" spans="1:10" ht="84.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
@@ -4797,7 +4809,7 @@
       <c r="I61" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="J61" s="35" t="s">
+      <c r="J61" s="18" t="s">
         <v>308</v>
       </c>
     </row>
@@ -4829,7 +4841,7 @@
       <c r="I62" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="J62" s="36" t="s">
+      <c r="J62" s="19" t="s">
         <v>313</v>
       </c>
     </row>
@@ -4840,13 +4852,13 @@
     <mergeCell ref="A11:J11"/>
     <mergeCell ref="A17:J17"/>
     <mergeCell ref="A20:J20"/>
+    <mergeCell ref="A57:J57"/>
+    <mergeCell ref="A60:J60"/>
     <mergeCell ref="A30:J30"/>
     <mergeCell ref="A35:J35"/>
     <mergeCell ref="A41:J41"/>
     <mergeCell ref="A46:J46"/>
     <mergeCell ref="A53:J53"/>
-    <mergeCell ref="A57:J57"/>
-    <mergeCell ref="A60:J60"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>